<commit_message>
Revert category forest plots + supp table to overall-model-p ordering
Order each panel (and the supp table) by the own-sex overall multivariate
Cox p-value, as before.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05_tcga_survival/motif_multivariate_TCGA/forest_by_TFcategory/SupplTable_TCGA_TFs_shared_unique.xlsx
+++ b/05_tcga_survival/motif_multivariate_TCGA/forest_by_TFcategory/SupplTable_TCGA_TFs_shared_unique.xlsx
@@ -62,12 +62,12 @@
     <t xml:space="preserve">KLF9</t>
   </si>
   <si>
+    <t xml:space="preserve">WT1</t>
+  </si>
+  <si>
     <t xml:space="preserve">ZFX</t>
   </si>
   <si>
-    <t xml:space="preserve">WT1</t>
-  </si>
-  <si>
     <t xml:space="preserve">KLF2</t>
   </si>
   <si>
@@ -86,12 +86,12 @@
     <t xml:space="preserve">EGR1</t>
   </si>
   <si>
+    <t xml:space="preserve">KLF15</t>
+  </si>
+  <si>
     <t xml:space="preserve">EGR3</t>
   </si>
   <si>
-    <t xml:space="preserve">KLF15</t>
-  </si>
-  <si>
     <t xml:space="preserve">ZNF263</t>
   </si>
   <si>
@@ -110,12 +110,12 @@
     <t xml:space="preserve">AHR</t>
   </si>
   <si>
+    <t xml:space="preserve">ARNT</t>
+  </si>
+  <si>
     <t xml:space="preserve">ZNF281</t>
   </si>
   <si>
-    <t xml:space="preserve">ARNT</t>
-  </si>
-  <si>
     <t xml:space="preserve">SP3</t>
   </si>
   <si>
@@ -134,52 +134,52 @@
     <t xml:space="preserve">Female-unique</t>
   </si>
   <si>
+    <t xml:space="preserve">ZIC1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KLF6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TCF7L1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TFAP2A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INSM1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUNX1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZNF682</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KLF3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THAP1</t>
+  </si>
+  <si>
     <t xml:space="preserve">TFAP2B</t>
   </si>
   <si>
+    <t xml:space="preserve">SOX15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KLF11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KLF10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RREB1</t>
+  </si>
+  <si>
     <t xml:space="preserve">PLAGL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KLF3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KLF6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOX15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZNF682</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TCF7L1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZIC1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KLF10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TFAP2A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KLF11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RUNX1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RREB1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INSM1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THAP1</t>
   </si>
 </sst>
 </file>
@@ -604,40 +604,40 @@
         <v>16</v>
       </c>
       <c r="C3" t="n">
-        <v>0.645</v>
+        <v>0.71</v>
       </c>
       <c r="D3" t="n">
-        <v>0.366</v>
+        <v>0.456</v>
       </c>
       <c r="E3" t="n">
-        <v>1.136</v>
+        <v>1.105</v>
       </c>
       <c r="F3" t="n">
         <v>0.129</v>
       </c>
       <c r="G3" t="n">
-        <v>1.867</v>
+        <v>1.349</v>
       </c>
       <c r="H3" t="n">
-        <v>1.128</v>
+        <v>1.053</v>
       </c>
       <c r="I3" t="n">
-        <v>3.09</v>
+        <v>1.729</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0152</v>
+        <v>0.0178</v>
       </c>
       <c r="K3" t="n">
-        <v>1.028</v>
+        <v>1.101</v>
       </c>
       <c r="L3" t="n">
-        <v>0.693</v>
+        <v>0.896</v>
       </c>
       <c r="M3" t="n">
-        <v>1.525</v>
+        <v>1.353</v>
       </c>
       <c r="N3" t="n">
-        <v>0.892</v>
+        <v>0.361</v>
       </c>
     </row>
     <row r="4">
@@ -648,40 +648,40 @@
         <v>17</v>
       </c>
       <c r="C4" t="n">
-        <v>0.71</v>
+        <v>0.645</v>
       </c>
       <c r="D4" t="n">
-        <v>0.456</v>
+        <v>0.366</v>
       </c>
       <c r="E4" t="n">
-        <v>1.105</v>
+        <v>1.136</v>
       </c>
       <c r="F4" t="n">
         <v>0.129</v>
       </c>
       <c r="G4" t="n">
-        <v>1.349</v>
+        <v>1.867</v>
       </c>
       <c r="H4" t="n">
-        <v>1.053</v>
+        <v>1.128</v>
       </c>
       <c r="I4" t="n">
-        <v>1.729</v>
+        <v>3.09</v>
       </c>
       <c r="J4" t="n">
-        <v>0.0178</v>
+        <v>0.0152</v>
       </c>
       <c r="K4" t="n">
-        <v>1.101</v>
+        <v>1.028</v>
       </c>
       <c r="L4" t="n">
-        <v>0.896</v>
+        <v>0.693</v>
       </c>
       <c r="M4" t="n">
-        <v>1.353</v>
+        <v>1.525</v>
       </c>
       <c r="N4" t="n">
-        <v>0.361</v>
+        <v>0.892</v>
       </c>
     </row>
     <row r="5">
@@ -912,40 +912,40 @@
         <v>24</v>
       </c>
       <c r="C10" t="n">
-        <v>1.195</v>
+        <v>0.401</v>
       </c>
       <c r="D10" t="n">
-        <v>1.032</v>
+        <v>0.188</v>
       </c>
       <c r="E10" t="n">
-        <v>1.385</v>
+        <v>0.855</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0176</v>
+        <v>0.018</v>
       </c>
       <c r="G10" t="n">
-        <v>0.928</v>
+        <v>5.493</v>
       </c>
       <c r="H10" t="n">
-        <v>0.755</v>
+        <v>1.824</v>
       </c>
       <c r="I10" t="n">
-        <v>1.141</v>
+        <v>16.539</v>
       </c>
       <c r="J10" t="n">
-        <v>0.477</v>
+        <v>0.00246</v>
       </c>
       <c r="K10" t="n">
-        <v>1.078</v>
+        <v>1.073</v>
       </c>
       <c r="L10" t="n">
-        <v>0.961</v>
+        <v>0.616</v>
       </c>
       <c r="M10" t="n">
-        <v>1.211</v>
+        <v>1.87</v>
       </c>
       <c r="N10" t="n">
-        <v>0.201</v>
+        <v>0.803</v>
       </c>
     </row>
     <row r="11">
@@ -956,40 +956,40 @@
         <v>25</v>
       </c>
       <c r="C11" t="n">
-        <v>0.401</v>
+        <v>1.195</v>
       </c>
       <c r="D11" t="n">
-        <v>0.188</v>
+        <v>1.032</v>
       </c>
       <c r="E11" t="n">
-        <v>0.855</v>
+        <v>1.385</v>
       </c>
       <c r="F11" t="n">
-        <v>0.018</v>
+        <v>0.0176</v>
       </c>
       <c r="G11" t="n">
-        <v>5.493</v>
+        <v>0.928</v>
       </c>
       <c r="H11" t="n">
-        <v>1.824</v>
+        <v>0.755</v>
       </c>
       <c r="I11" t="n">
-        <v>16.539</v>
+        <v>1.141</v>
       </c>
       <c r="J11" t="n">
-        <v>0.00246</v>
+        <v>0.477</v>
       </c>
       <c r="K11" t="n">
-        <v>1.073</v>
+        <v>1.078</v>
       </c>
       <c r="L11" t="n">
-        <v>0.616</v>
+        <v>0.961</v>
       </c>
       <c r="M11" t="n">
-        <v>1.87</v>
+        <v>1.211</v>
       </c>
       <c r="N11" t="n">
-        <v>0.803</v>
+        <v>0.201</v>
       </c>
     </row>
     <row r="12">
@@ -1264,40 +1264,40 @@
         <v>32</v>
       </c>
       <c r="C18" t="n">
-        <v>0.844</v>
+        <v>0.805</v>
       </c>
       <c r="D18" t="n">
-        <v>0.557</v>
+        <v>0.471</v>
       </c>
       <c r="E18" t="n">
-        <v>1.278</v>
+        <v>1.375</v>
       </c>
       <c r="F18" t="n">
-        <v>0.423</v>
+        <v>0.426</v>
       </c>
       <c r="G18" t="n">
-        <v>1.354</v>
+        <v>1.569</v>
       </c>
       <c r="H18" t="n">
-        <v>0.887</v>
+        <v>0.804</v>
       </c>
       <c r="I18" t="n">
-        <v>2.067</v>
+        <v>3.064</v>
       </c>
       <c r="J18" t="n">
-        <v>0.16</v>
+        <v>0.187</v>
       </c>
       <c r="K18" t="n">
-        <v>1.063</v>
+        <v>1.051</v>
       </c>
       <c r="L18" t="n">
-        <v>0.802</v>
+        <v>0.698</v>
       </c>
       <c r="M18" t="n">
-        <v>1.409</v>
+        <v>1.583</v>
       </c>
       <c r="N18" t="n">
-        <v>0.672</v>
+        <v>0.812</v>
       </c>
     </row>
     <row r="19">
@@ -1308,40 +1308,40 @@
         <v>33</v>
       </c>
       <c r="C19" t="n">
-        <v>0.805</v>
+        <v>0.844</v>
       </c>
       <c r="D19" t="n">
-        <v>0.471</v>
+        <v>0.557</v>
       </c>
       <c r="E19" t="n">
-        <v>1.375</v>
+        <v>1.278</v>
       </c>
       <c r="F19" t="n">
-        <v>0.426</v>
+        <v>0.423</v>
       </c>
       <c r="G19" t="n">
-        <v>1.569</v>
+        <v>1.354</v>
       </c>
       <c r="H19" t="n">
-        <v>0.804</v>
+        <v>0.887</v>
       </c>
       <c r="I19" t="n">
-        <v>3.064</v>
+        <v>2.067</v>
       </c>
       <c r="J19" t="n">
-        <v>0.187</v>
+        <v>0.16</v>
       </c>
       <c r="K19" t="n">
-        <v>1.051</v>
+        <v>1.063</v>
       </c>
       <c r="L19" t="n">
-        <v>0.698</v>
+        <v>0.802</v>
       </c>
       <c r="M19" t="n">
-        <v>1.583</v>
+        <v>1.409</v>
       </c>
       <c r="N19" t="n">
-        <v>0.812</v>
+        <v>0.672</v>
       </c>
     </row>
     <row r="20">
@@ -1572,40 +1572,40 @@
         <v>40</v>
       </c>
       <c r="C25" t="n">
-        <v>0.569</v>
+        <v>1.05</v>
       </c>
       <c r="D25" t="n">
-        <v>0.33</v>
+        <v>0.932</v>
       </c>
       <c r="E25" t="n">
-        <v>0.979</v>
+        <v>1.184</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0419</v>
+        <v>0.423</v>
       </c>
       <c r="G25" t="n">
-        <v>0.81</v>
+        <v>0.812</v>
       </c>
       <c r="H25" t="n">
-        <v>0.403</v>
+        <v>0.72</v>
       </c>
       <c r="I25" t="n">
-        <v>1.628</v>
+        <v>0.916</v>
       </c>
       <c r="J25" t="n">
-        <v>0.553</v>
+        <v>0.000702</v>
       </c>
       <c r="K25" t="n">
-        <v>0.709</v>
+        <v>0.912</v>
       </c>
       <c r="L25" t="n">
-        <v>0.474</v>
+        <v>0.84</v>
       </c>
       <c r="M25" t="n">
-        <v>1.061</v>
+        <v>0.99</v>
       </c>
       <c r="N25" t="n">
-        <v>0.0948</v>
+        <v>0.0269</v>
       </c>
     </row>
     <row r="26">
@@ -1616,40 +1616,40 @@
         <v>41</v>
       </c>
       <c r="C26" t="n">
-        <v>0.807</v>
+        <v>0.808</v>
       </c>
       <c r="D26" t="n">
-        <v>0.65</v>
+        <v>0.485</v>
       </c>
       <c r="E26" t="n">
-        <v>1.003</v>
+        <v>1.343</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0528</v>
+        <v>0.411</v>
       </c>
       <c r="G26" t="n">
-        <v>1.001</v>
+        <v>0.489</v>
       </c>
       <c r="H26" t="n">
-        <v>0.798</v>
+        <v>0.295</v>
       </c>
       <c r="I26" t="n">
-        <v>1.257</v>
+        <v>0.812</v>
       </c>
       <c r="J26" t="n">
-        <v>0.991</v>
+        <v>0.00567</v>
       </c>
       <c r="K26" t="n">
-        <v>0.927</v>
+        <v>0.62</v>
       </c>
       <c r="L26" t="n">
-        <v>0.805</v>
+        <v>0.441</v>
       </c>
       <c r="M26" t="n">
-        <v>1.068</v>
+        <v>0.874</v>
       </c>
       <c r="N26" t="n">
-        <v>0.295</v>
+        <v>0.00625</v>
       </c>
     </row>
     <row r="27">
@@ -1660,40 +1660,40 @@
         <v>42</v>
       </c>
       <c r="C27" t="n">
-        <v>1.443</v>
+        <v>1.175</v>
       </c>
       <c r="D27" t="n">
-        <v>0.952</v>
+        <v>0.953</v>
       </c>
       <c r="E27" t="n">
-        <v>2.186</v>
+        <v>1.449</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0836</v>
+        <v>0.132</v>
       </c>
       <c r="G27" t="n">
-        <v>1.281</v>
+        <v>1.519</v>
       </c>
       <c r="H27" t="n">
-        <v>0.746</v>
+        <v>1.143</v>
       </c>
       <c r="I27" t="n">
-        <v>2.201</v>
+        <v>2.02</v>
       </c>
       <c r="J27" t="n">
-        <v>0.369</v>
+        <v>0.00402</v>
       </c>
       <c r="K27" t="n">
-        <v>1.155</v>
+        <v>1.327</v>
       </c>
       <c r="L27" t="n">
-        <v>0.837</v>
+        <v>1.121</v>
       </c>
       <c r="M27" t="n">
-        <v>1.593</v>
+        <v>1.571</v>
       </c>
       <c r="N27" t="n">
-        <v>0.382</v>
+        <v>0.000986</v>
       </c>
     </row>
     <row r="28">
@@ -1704,40 +1704,40 @@
         <v>43</v>
       </c>
       <c r="C28" t="n">
-        <v>1.175</v>
+        <v>1.144</v>
       </c>
       <c r="D28" t="n">
-        <v>0.953</v>
+        <v>0.921</v>
       </c>
       <c r="E28" t="n">
-        <v>1.449</v>
+        <v>1.421</v>
       </c>
       <c r="F28" t="n">
-        <v>0.132</v>
+        <v>0.225</v>
       </c>
       <c r="G28" t="n">
-        <v>1.519</v>
+        <v>0.744</v>
       </c>
       <c r="H28" t="n">
-        <v>1.143</v>
+        <v>0.586</v>
       </c>
       <c r="I28" t="n">
-        <v>2.02</v>
+        <v>0.945</v>
       </c>
       <c r="J28" t="n">
-        <v>0.00402</v>
+        <v>0.0154</v>
       </c>
       <c r="K28" t="n">
-        <v>1.327</v>
+        <v>0.92</v>
       </c>
       <c r="L28" t="n">
-        <v>1.121</v>
+        <v>0.793</v>
       </c>
       <c r="M28" t="n">
-        <v>1.571</v>
+        <v>1.067</v>
       </c>
       <c r="N28" t="n">
-        <v>0.000986</v>
+        <v>0.268</v>
       </c>
     </row>
     <row r="29">
@@ -1748,40 +1748,40 @@
         <v>44</v>
       </c>
       <c r="C29" t="n">
-        <v>0.781</v>
+        <v>1.049</v>
       </c>
       <c r="D29" t="n">
-        <v>0.538</v>
+        <v>0.765</v>
       </c>
       <c r="E29" t="n">
-        <v>1.133</v>
+        <v>1.439</v>
       </c>
       <c r="F29" t="n">
-        <v>0.192</v>
+        <v>0.766</v>
       </c>
       <c r="G29" t="n">
-        <v>0.916</v>
+        <v>1.286</v>
       </c>
       <c r="H29" t="n">
-        <v>0.619</v>
+        <v>0.959</v>
       </c>
       <c r="I29" t="n">
-        <v>1.356</v>
+        <v>1.725</v>
       </c>
       <c r="J29" t="n">
-        <v>0.662</v>
+        <v>0.0929</v>
       </c>
       <c r="K29" t="n">
-        <v>0.86</v>
+        <v>1.19</v>
       </c>
       <c r="L29" t="n">
-        <v>0.667</v>
+        <v>0.976</v>
       </c>
       <c r="M29" t="n">
-        <v>1.108</v>
+        <v>1.452</v>
       </c>
       <c r="N29" t="n">
-        <v>0.243</v>
+        <v>0.0856</v>
       </c>
     </row>
     <row r="30">
@@ -1792,40 +1792,40 @@
         <v>45</v>
       </c>
       <c r="C30" t="n">
-        <v>1.411</v>
+        <v>0.993</v>
       </c>
       <c r="D30" t="n">
-        <v>0.811</v>
+        <v>0.885</v>
       </c>
       <c r="E30" t="n">
-        <v>2.455</v>
+        <v>1.113</v>
       </c>
       <c r="F30" t="n">
-        <v>0.223</v>
+        <v>0.899</v>
       </c>
       <c r="G30" t="n">
-        <v>0.668</v>
+        <v>0.906</v>
       </c>
       <c r="H30" t="n">
-        <v>0.302</v>
+        <v>0.786</v>
       </c>
       <c r="I30" t="n">
-        <v>1.477</v>
+        <v>1.044</v>
       </c>
       <c r="J30" t="n">
-        <v>0.318</v>
+        <v>0.172</v>
       </c>
       <c r="K30" t="n">
-        <v>0.982</v>
+        <v>0.964</v>
       </c>
       <c r="L30" t="n">
-        <v>0.631</v>
+        <v>0.883</v>
       </c>
       <c r="M30" t="n">
-        <v>1.529</v>
+        <v>1.052</v>
       </c>
       <c r="N30" t="n">
-        <v>0.937</v>
+        <v>0.413</v>
       </c>
     </row>
     <row r="31">
@@ -1836,40 +1836,40 @@
         <v>46</v>
       </c>
       <c r="C31" t="n">
-        <v>1.144</v>
+        <v>0.853</v>
       </c>
       <c r="D31" t="n">
-        <v>0.921</v>
+        <v>0.254</v>
       </c>
       <c r="E31" t="n">
-        <v>1.421</v>
+        <v>2.868</v>
       </c>
       <c r="F31" t="n">
-        <v>0.225</v>
+        <v>0.797</v>
       </c>
       <c r="G31" t="n">
-        <v>0.744</v>
+        <v>3.139</v>
       </c>
       <c r="H31" t="n">
-        <v>0.586</v>
+        <v>0.6</v>
       </c>
       <c r="I31" t="n">
-        <v>0.945</v>
+        <v>16.408</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0154</v>
+        <v>0.175</v>
       </c>
       <c r="K31" t="n">
-        <v>0.92</v>
+        <v>1.118</v>
       </c>
       <c r="L31" t="n">
-        <v>0.793</v>
+        <v>0.428</v>
       </c>
       <c r="M31" t="n">
-        <v>1.067</v>
+        <v>2.918</v>
       </c>
       <c r="N31" t="n">
-        <v>0.268</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="32">
@@ -1880,40 +1880,40 @@
         <v>47</v>
       </c>
       <c r="C32" t="n">
-        <v>0.808</v>
+        <v>1.411</v>
       </c>
       <c r="D32" t="n">
-        <v>0.485</v>
+        <v>0.811</v>
       </c>
       <c r="E32" t="n">
-        <v>1.343</v>
+        <v>2.455</v>
       </c>
       <c r="F32" t="n">
-        <v>0.411</v>
+        <v>0.223</v>
       </c>
       <c r="G32" t="n">
-        <v>0.489</v>
+        <v>0.668</v>
       </c>
       <c r="H32" t="n">
-        <v>0.295</v>
+        <v>0.302</v>
       </c>
       <c r="I32" t="n">
-        <v>0.812</v>
+        <v>1.477</v>
       </c>
       <c r="J32" t="n">
-        <v>0.00567</v>
+        <v>0.318</v>
       </c>
       <c r="K32" t="n">
-        <v>0.62</v>
+        <v>0.982</v>
       </c>
       <c r="L32" t="n">
-        <v>0.441</v>
+        <v>0.631</v>
       </c>
       <c r="M32" t="n">
-        <v>0.874</v>
+        <v>1.529</v>
       </c>
       <c r="N32" t="n">
-        <v>0.00625</v>
+        <v>0.937</v>
       </c>
     </row>
     <row r="33">
@@ -1924,40 +1924,40 @@
         <v>48</v>
       </c>
       <c r="C33" t="n">
-        <v>1.05</v>
+        <v>1.443</v>
       </c>
       <c r="D33" t="n">
-        <v>0.932</v>
+        <v>0.952</v>
       </c>
       <c r="E33" t="n">
-        <v>1.184</v>
+        <v>2.186</v>
       </c>
       <c r="F33" t="n">
-        <v>0.423</v>
+        <v>0.0836</v>
       </c>
       <c r="G33" t="n">
-        <v>0.812</v>
+        <v>1.281</v>
       </c>
       <c r="H33" t="n">
-        <v>0.72</v>
+        <v>0.746</v>
       </c>
       <c r="I33" t="n">
-        <v>0.916</v>
+        <v>2.201</v>
       </c>
       <c r="J33" t="n">
-        <v>0.000702</v>
+        <v>0.369</v>
       </c>
       <c r="K33" t="n">
-        <v>0.912</v>
+        <v>1.155</v>
       </c>
       <c r="L33" t="n">
-        <v>0.84</v>
+        <v>0.837</v>
       </c>
       <c r="M33" t="n">
-        <v>0.99</v>
+        <v>1.593</v>
       </c>
       <c r="N33" t="n">
-        <v>0.0269</v>
+        <v>0.382</v>
       </c>
     </row>
     <row r="34">
@@ -1968,40 +1968,40 @@
         <v>49</v>
       </c>
       <c r="C34" t="n">
-        <v>1.095</v>
+        <v>1.004</v>
       </c>
       <c r="D34" t="n">
-        <v>0.795</v>
+        <v>0.664</v>
       </c>
       <c r="E34" t="n">
-        <v>1.508</v>
+        <v>1.519</v>
       </c>
       <c r="F34" t="n">
-        <v>0.58</v>
+        <v>0.985</v>
       </c>
       <c r="G34" t="n">
-        <v>1.028</v>
+        <v>0.834</v>
       </c>
       <c r="H34" t="n">
-        <v>0.703</v>
+        <v>0.554</v>
       </c>
       <c r="I34" t="n">
-        <v>1.504</v>
+        <v>1.256</v>
       </c>
       <c r="J34" t="n">
-        <v>0.886</v>
+        <v>0.385</v>
       </c>
       <c r="K34" t="n">
-        <v>1.024</v>
+        <v>0.935</v>
       </c>
       <c r="L34" t="n">
-        <v>0.807</v>
+        <v>0.714</v>
       </c>
       <c r="M34" t="n">
-        <v>1.3</v>
+        <v>1.225</v>
       </c>
       <c r="N34" t="n">
-        <v>0.843</v>
+        <v>0.626</v>
       </c>
     </row>
     <row r="35">
@@ -2012,40 +2012,40 @@
         <v>50</v>
       </c>
       <c r="C35" t="n">
-        <v>1.049</v>
+        <v>0.569</v>
       </c>
       <c r="D35" t="n">
-        <v>0.765</v>
+        <v>0.33</v>
       </c>
       <c r="E35" t="n">
-        <v>1.439</v>
+        <v>0.979</v>
       </c>
       <c r="F35" t="n">
-        <v>0.766</v>
+        <v>0.0419</v>
       </c>
       <c r="G35" t="n">
-        <v>1.286</v>
+        <v>0.81</v>
       </c>
       <c r="H35" t="n">
-        <v>0.959</v>
+        <v>0.403</v>
       </c>
       <c r="I35" t="n">
-        <v>1.725</v>
+        <v>1.628</v>
       </c>
       <c r="J35" t="n">
-        <v>0.0929</v>
+        <v>0.553</v>
       </c>
       <c r="K35" t="n">
-        <v>1.19</v>
+        <v>0.709</v>
       </c>
       <c r="L35" t="n">
-        <v>0.976</v>
+        <v>0.474</v>
       </c>
       <c r="M35" t="n">
-        <v>1.452</v>
+        <v>1.061</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0856</v>
+        <v>0.0948</v>
       </c>
     </row>
     <row r="36">
@@ -2056,40 +2056,40 @@
         <v>51</v>
       </c>
       <c r="C36" t="n">
-        <v>0.958</v>
+        <v>0.781</v>
       </c>
       <c r="D36" t="n">
-        <v>0.717</v>
+        <v>0.538</v>
       </c>
       <c r="E36" t="n">
-        <v>1.28</v>
+        <v>1.133</v>
       </c>
       <c r="F36" t="n">
-        <v>0.77</v>
+        <v>0.192</v>
       </c>
       <c r="G36" t="n">
-        <v>1.063</v>
+        <v>0.916</v>
       </c>
       <c r="H36" t="n">
-        <v>0.775</v>
+        <v>0.619</v>
       </c>
       <c r="I36" t="n">
-        <v>1.458</v>
+        <v>1.356</v>
       </c>
       <c r="J36" t="n">
-        <v>0.706</v>
+        <v>0.662</v>
       </c>
       <c r="K36" t="n">
-        <v>0.984</v>
+        <v>0.86</v>
       </c>
       <c r="L36" t="n">
-        <v>0.799</v>
+        <v>0.667</v>
       </c>
       <c r="M36" t="n">
-        <v>1.211</v>
+        <v>1.108</v>
       </c>
       <c r="N36" t="n">
-        <v>0.877</v>
+        <v>0.243</v>
       </c>
     </row>
     <row r="37">
@@ -2100,40 +2100,40 @@
         <v>52</v>
       </c>
       <c r="C37" t="n">
-        <v>0.853</v>
+        <v>0.958</v>
       </c>
       <c r="D37" t="n">
-        <v>0.254</v>
+        <v>0.717</v>
       </c>
       <c r="E37" t="n">
-        <v>2.868</v>
+        <v>1.28</v>
       </c>
       <c r="F37" t="n">
-        <v>0.797</v>
+        <v>0.77</v>
       </c>
       <c r="G37" t="n">
-        <v>3.139</v>
+        <v>1.063</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6</v>
+        <v>0.775</v>
       </c>
       <c r="I37" t="n">
-        <v>16.408</v>
+        <v>1.458</v>
       </c>
       <c r="J37" t="n">
-        <v>0.175</v>
+        <v>0.706</v>
       </c>
       <c r="K37" t="n">
-        <v>1.118</v>
+        <v>0.984</v>
       </c>
       <c r="L37" t="n">
-        <v>0.428</v>
+        <v>0.799</v>
       </c>
       <c r="M37" t="n">
-        <v>2.918</v>
+        <v>1.211</v>
       </c>
       <c r="N37" t="n">
-        <v>0.82</v>
+        <v>0.877</v>
       </c>
     </row>
     <row r="38">
@@ -2144,40 +2144,40 @@
         <v>53</v>
       </c>
       <c r="C38" t="n">
-        <v>1.118</v>
+        <v>1.095</v>
       </c>
       <c r="D38" t="n">
-        <v>0.377</v>
+        <v>0.795</v>
       </c>
       <c r="E38" t="n">
-        <v>3.319</v>
+        <v>1.508</v>
       </c>
       <c r="F38" t="n">
-        <v>0.841</v>
+        <v>0.58</v>
       </c>
       <c r="G38" t="n">
-        <v>1.021</v>
+        <v>1.028</v>
       </c>
       <c r="H38" t="n">
-        <v>0.236</v>
+        <v>0.703</v>
       </c>
       <c r="I38" t="n">
-        <v>4.417</v>
+        <v>1.504</v>
       </c>
       <c r="J38" t="n">
-        <v>0.978</v>
+        <v>0.886</v>
       </c>
       <c r="K38" t="n">
-        <v>0.944</v>
+        <v>1.024</v>
       </c>
       <c r="L38" t="n">
-        <v>0.397</v>
+        <v>0.807</v>
       </c>
       <c r="M38" t="n">
-        <v>2.247</v>
+        <v>1.3</v>
       </c>
       <c r="N38" t="n">
-        <v>0.897</v>
+        <v>0.843</v>
       </c>
     </row>
     <row r="39">
@@ -2188,40 +2188,40 @@
         <v>54</v>
       </c>
       <c r="C39" t="n">
-        <v>0.993</v>
+        <v>1.118</v>
       </c>
       <c r="D39" t="n">
-        <v>0.885</v>
+        <v>0.377</v>
       </c>
       <c r="E39" t="n">
-        <v>1.113</v>
+        <v>3.319</v>
       </c>
       <c r="F39" t="n">
-        <v>0.899</v>
+        <v>0.841</v>
       </c>
       <c r="G39" t="n">
-        <v>0.906</v>
+        <v>1.021</v>
       </c>
       <c r="H39" t="n">
-        <v>0.786</v>
+        <v>0.236</v>
       </c>
       <c r="I39" t="n">
-        <v>1.044</v>
+        <v>4.417</v>
       </c>
       <c r="J39" t="n">
-        <v>0.172</v>
+        <v>0.978</v>
       </c>
       <c r="K39" t="n">
-        <v>0.964</v>
+        <v>0.944</v>
       </c>
       <c r="L39" t="n">
-        <v>0.883</v>
+        <v>0.397</v>
       </c>
       <c r="M39" t="n">
-        <v>1.052</v>
+        <v>2.247</v>
       </c>
       <c r="N39" t="n">
-        <v>0.413</v>
+        <v>0.897</v>
       </c>
     </row>
     <row r="40">
@@ -2232,40 +2232,40 @@
         <v>55</v>
       </c>
       <c r="C40" t="n">
-        <v>1.004</v>
+        <v>0.807</v>
       </c>
       <c r="D40" t="n">
-        <v>0.664</v>
+        <v>0.65</v>
       </c>
       <c r="E40" t="n">
-        <v>1.519</v>
+        <v>1.003</v>
       </c>
       <c r="F40" t="n">
-        <v>0.985</v>
+        <v>0.0528</v>
       </c>
       <c r="G40" t="n">
-        <v>0.834</v>
+        <v>1.001</v>
       </c>
       <c r="H40" t="n">
-        <v>0.554</v>
+        <v>0.798</v>
       </c>
       <c r="I40" t="n">
-        <v>1.256</v>
+        <v>1.257</v>
       </c>
       <c r="J40" t="n">
-        <v>0.385</v>
+        <v>0.991</v>
       </c>
       <c r="K40" t="n">
-        <v>0.935</v>
+        <v>0.927</v>
       </c>
       <c r="L40" t="n">
-        <v>0.714</v>
+        <v>0.805</v>
       </c>
       <c r="M40" t="n">
-        <v>1.225</v>
+        <v>1.068</v>
       </c>
       <c r="N40" t="n">
-        <v>0.626</v>
+        <v>0.295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>